<commit_message>
checkpoint: 2026-07-21 08:57 (auto)
</commit_message>
<xml_diff>
--- a/pl_tracker.xlsx
+++ b/pl_tracker.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -437,7 +437,7 @@
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -530,6 +530,23 @@
       <c r="G2" t="n">
         <v>34940.29</v>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>262.83</v>
+      </c>
+      <c r="J2" t="n">
+        <v>35482.05</v>
+      </c>
+      <c r="K2" t="n">
+        <v>-541.76</v>
+      </c>
+      <c r="L2" t="n">
+        <v>-0.015505</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -559,6 +576,23 @@
       <c r="G3" t="n">
         <v>34902</v>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>85.08</v>
+      </c>
+      <c r="J3" t="n">
+        <v>35733.6</v>
+      </c>
+      <c r="K3" t="n">
+        <v>831.6</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.023827</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -588,6 +622,23 @@
       <c r="G4" t="n">
         <v>34858.72</v>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>83.28</v>
+      </c>
+      <c r="J4" t="n">
+        <v>34644.48</v>
+      </c>
+      <c r="K4" t="n">
+        <v>-214.24</v>
+      </c>
+      <c r="L4" t="n">
+        <v>-0.006146</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -617,6 +668,23 @@
       <c r="G5" t="n">
         <v>34854.03</v>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>415.71</v>
+      </c>
+      <c r="J5" t="n">
+        <v>36166.77</v>
+      </c>
+      <c r="K5" t="n">
+        <v>-1312.74</v>
+      </c>
+      <c r="L5" t="n">
+        <v>-0.037664</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -646,6 +714,23 @@
       <c r="G6" t="n">
         <v>34791.84</v>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>119.1</v>
+      </c>
+      <c r="J6" t="n">
+        <v>35253.6</v>
+      </c>
+      <c r="K6" t="n">
+        <v>461.76</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.013272</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -674,6 +759,2129 @@
       </c>
       <c r="G7" t="n">
         <v>34967.71</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>154.35</v>
+      </c>
+      <c r="J7" t="n">
+        <v>35963.55</v>
+      </c>
+      <c r="K7" t="n">
+        <v>-995.84</v>
+      </c>
+      <c r="L7" t="n">
+        <v>-0.028479</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>XLB</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>666</v>
+      </c>
+      <c r="F8" t="n">
+        <v>51.88</v>
+      </c>
+      <c r="G8" t="n">
+        <v>34552.08</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>51.92</v>
+      </c>
+      <c r="J8" t="n">
+        <v>34578.72</v>
+      </c>
+      <c r="K8" t="n">
+        <v>26.64</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.000771</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>IYT</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>422</v>
+      </c>
+      <c r="F9" t="n">
+        <v>81.87</v>
+      </c>
+      <c r="G9" t="n">
+        <v>34549.14</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>81.34999999999999</v>
+      </c>
+      <c r="J9" t="n">
+        <v>34329.7</v>
+      </c>
+      <c r="K9" t="n">
+        <v>-219.44</v>
+      </c>
+      <c r="L9" t="n">
+        <v>-0.006352</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>IGV</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>406</v>
+      </c>
+      <c r="F10" t="n">
+        <v>85.08</v>
+      </c>
+      <c r="G10" t="n">
+        <v>34542.48</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>85.2</v>
+      </c>
+      <c r="J10" t="n">
+        <v>34591.2</v>
+      </c>
+      <c r="K10" t="n">
+        <v>48.72</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.00141</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>XBI</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>249</v>
+      </c>
+      <c r="F11" t="n">
+        <v>138.67</v>
+      </c>
+      <c r="G11" t="n">
+        <v>34528.83</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>133.28</v>
+      </c>
+      <c r="J11" t="n">
+        <v>33186.72</v>
+      </c>
+      <c r="K11" t="n">
+        <v>1342.11</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.038869</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>SMH</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>74</v>
+      </c>
+      <c r="F12" t="n">
+        <v>464.16</v>
+      </c>
+      <c r="G12" t="n">
+        <v>34347.84</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>506.44</v>
+      </c>
+      <c r="J12" t="n">
+        <v>37476.56</v>
+      </c>
+      <c r="K12" t="n">
+        <v>-3128.72</v>
+      </c>
+      <c r="L12" t="n">
+        <v>-0.091089</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>83</v>
+      </c>
+      <c r="F13" t="n">
+        <v>415.71</v>
+      </c>
+      <c r="G13" t="n">
+        <v>34503.93</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>461.6</v>
+      </c>
+      <c r="J13" t="n">
+        <v>38312.8</v>
+      </c>
+      <c r="K13" t="n">
+        <v>-3808.87</v>
+      </c>
+      <c r="L13" t="n">
+        <v>-0.110389</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>XBI</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>252</v>
+      </c>
+      <c r="F14" t="n">
+        <v>133.28</v>
+      </c>
+      <c r="G14" t="n">
+        <v>33586.56</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>130.42</v>
+      </c>
+      <c r="J14" t="n">
+        <v>32865.84</v>
+      </c>
+      <c r="K14" t="n">
+        <v>-720.72</v>
+      </c>
+      <c r="L14" t="n">
+        <v>-0.021459</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>3</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>IHI</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>637</v>
+      </c>
+      <c r="F15" t="n">
+        <v>52.81</v>
+      </c>
+      <c r="G15" t="n">
+        <v>33639.97</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="J15" t="n">
+        <v>32168.5</v>
+      </c>
+      <c r="K15" t="n">
+        <v>-1471.47</v>
+      </c>
+      <c r="L15" t="n">
+        <v>-0.043742</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>KBE</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>530</v>
+      </c>
+      <c r="F16" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="G16" t="n">
+        <v>33655</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>64.06999999999999</v>
+      </c>
+      <c r="J16" t="n">
+        <v>33957.1</v>
+      </c>
+      <c r="K16" t="n">
+        <v>302.1</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.008976</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>3</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>XLK</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>210</v>
+      </c>
+      <c r="F17" t="n">
+        <v>160.22</v>
+      </c>
+      <c r="G17" t="n">
+        <v>33646.2</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>161.87</v>
+      </c>
+      <c r="J17" t="n">
+        <v>33992.7</v>
+      </c>
+      <c r="K17" t="n">
+        <v>-346.5</v>
+      </c>
+      <c r="L17" t="n">
+        <v>-0.010298</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>SMH</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>66</v>
+      </c>
+      <c r="F18" t="n">
+        <v>506.44</v>
+      </c>
+      <c r="G18" t="n">
+        <v>33425.04</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>509.82</v>
+      </c>
+      <c r="J18" t="n">
+        <v>33648.12</v>
+      </c>
+      <c r="K18" t="n">
+        <v>-223.08</v>
+      </c>
+      <c r="L18" t="n">
+        <v>-0.006674</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>3</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>72</v>
+      </c>
+      <c r="F19" t="n">
+        <v>461.6</v>
+      </c>
+      <c r="G19" t="n">
+        <v>33235.2</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>465.75</v>
+      </c>
+      <c r="J19" t="n">
+        <v>33534</v>
+      </c>
+      <c r="K19" t="n">
+        <v>-298.8</v>
+      </c>
+      <c r="L19" t="n">
+        <v>-0.00899</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>4</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>IHI</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>667</v>
+      </c>
+      <c r="F20" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="G20" t="n">
+        <v>33683.5</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>49.01</v>
+      </c>
+      <c r="J20" t="n">
+        <v>32689.67</v>
+      </c>
+      <c r="K20" t="n">
+        <v>-993.83</v>
+      </c>
+      <c r="L20" t="n">
+        <v>-0.029505</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>ITB</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>355</v>
+      </c>
+      <c r="F21" t="n">
+        <v>94.84</v>
+      </c>
+      <c r="G21" t="n">
+        <v>33668.2</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>93</v>
+      </c>
+      <c r="J21" t="n">
+        <v>33015</v>
+      </c>
+      <c r="K21" t="n">
+        <v>-653.2</v>
+      </c>
+      <c r="L21" t="n">
+        <v>-0.019401</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>4</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>XLB</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>656</v>
+      </c>
+      <c r="F22" t="n">
+        <v>51.35</v>
+      </c>
+      <c r="G22" t="n">
+        <v>33685.6</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>51.59</v>
+      </c>
+      <c r="J22" t="n">
+        <v>33843.04</v>
+      </c>
+      <c r="K22" t="n">
+        <v>157.44</v>
+      </c>
+      <c r="L22" t="n">
+        <v>0.004674</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>4</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>OIH</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>75</v>
+      </c>
+      <c r="F23" t="n">
+        <v>444.73</v>
+      </c>
+      <c r="G23" t="n">
+        <v>33354.75</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>420.84</v>
+      </c>
+      <c r="J23" t="n">
+        <v>31563</v>
+      </c>
+      <c r="K23" t="n">
+        <v>1791.75</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0.053718</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>4</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>72</v>
+      </c>
+      <c r="F24" t="n">
+        <v>465.75</v>
+      </c>
+      <c r="G24" t="n">
+        <v>33534</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>520.3</v>
+      </c>
+      <c r="J24" t="n">
+        <v>37461.6</v>
+      </c>
+      <c r="K24" t="n">
+        <v>-3927.6</v>
+      </c>
+      <c r="L24" t="n">
+        <v>-0.117123</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>4</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>FDN</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>126</v>
+      </c>
+      <c r="F25" t="n">
+        <v>266.11</v>
+      </c>
+      <c r="G25" t="n">
+        <v>33529.86</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>267.6</v>
+      </c>
+      <c r="J25" t="n">
+        <v>33717.6</v>
+      </c>
+      <c r="K25" t="n">
+        <v>-187.74</v>
+      </c>
+      <c r="L25" t="n">
+        <v>-0.005599</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>5</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>IHI</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>674</v>
+      </c>
+      <c r="F26" t="n">
+        <v>49.01</v>
+      </c>
+      <c r="G26" t="n">
+        <v>33032.74</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>48.46</v>
+      </c>
+      <c r="J26" t="n">
+        <v>32662.04</v>
+      </c>
+      <c r="K26" t="n">
+        <v>-370.7</v>
+      </c>
+      <c r="L26" t="n">
+        <v>-0.011222</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>5</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>KBE</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>515</v>
+      </c>
+      <c r="F27" t="n">
+        <v>64.05</v>
+      </c>
+      <c r="G27" t="n">
+        <v>32985.75</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>61.68</v>
+      </c>
+      <c r="J27" t="n">
+        <v>31765.2</v>
+      </c>
+      <c r="K27" t="n">
+        <v>-1220.55</v>
+      </c>
+      <c r="L27" t="n">
+        <v>-0.037002</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>5</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>XLV</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>230</v>
+      </c>
+      <c r="F28" t="n">
+        <v>143.49</v>
+      </c>
+      <c r="G28" t="n">
+        <v>33002.7</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>145.1</v>
+      </c>
+      <c r="J28" t="n">
+        <v>33373</v>
+      </c>
+      <c r="K28" t="n">
+        <v>370.3</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0.01122</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>5</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>IGV</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>362</v>
+      </c>
+      <c r="F29" t="n">
+        <v>91.15000000000001</v>
+      </c>
+      <c r="G29" t="n">
+        <v>32996.3</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>91.78</v>
+      </c>
+      <c r="J29" t="n">
+        <v>33224.36</v>
+      </c>
+      <c r="K29" t="n">
+        <v>-228.06</v>
+      </c>
+      <c r="L29" t="n">
+        <v>-0.006912</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>5</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>63</v>
+      </c>
+      <c r="F30" t="n">
+        <v>520.3</v>
+      </c>
+      <c r="G30" t="n">
+        <v>32778.9</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>508.52</v>
+      </c>
+      <c r="J30" t="n">
+        <v>32036.76</v>
+      </c>
+      <c r="K30" t="n">
+        <v>742.14</v>
+      </c>
+      <c r="L30" t="n">
+        <v>0.022641</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>5</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>SMH</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>58</v>
+      </c>
+      <c r="F31" t="n">
+        <v>566.54</v>
+      </c>
+      <c r="G31" t="n">
+        <v>32859.32</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>556.34</v>
+      </c>
+      <c r="J31" t="n">
+        <v>32267.72</v>
+      </c>
+      <c r="K31" t="n">
+        <v>591.6</v>
+      </c>
+      <c r="L31" t="n">
+        <v>0.018004</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>6</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ITB</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>382</v>
+      </c>
+      <c r="F32" t="n">
+        <v>86.45</v>
+      </c>
+      <c r="G32" t="n">
+        <v>33023.9</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>93.06</v>
+      </c>
+      <c r="J32" t="n">
+        <v>35548.92</v>
+      </c>
+      <c r="K32" t="n">
+        <v>2525.02</v>
+      </c>
+      <c r="L32" t="n">
+        <v>0.07646</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>6</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>IHI</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>681</v>
+      </c>
+      <c r="F33" t="n">
+        <v>48.46</v>
+      </c>
+      <c r="G33" t="n">
+        <v>33001.26</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>48.96</v>
+      </c>
+      <c r="J33" t="n">
+        <v>33341.76</v>
+      </c>
+      <c r="K33" t="n">
+        <v>340.5</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0.010318</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>6</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>XLRE</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>764</v>
+      </c>
+      <c r="F34" t="n">
+        <v>43.23</v>
+      </c>
+      <c r="G34" t="n">
+        <v>33027.72</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>43.99</v>
+      </c>
+      <c r="J34" t="n">
+        <v>33608.36</v>
+      </c>
+      <c r="K34" t="n">
+        <v>580.64</v>
+      </c>
+      <c r="L34" t="n">
+        <v>0.01758</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>6</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>XLY</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>283</v>
+      </c>
+      <c r="F35" t="n">
+        <v>116.53</v>
+      </c>
+      <c r="G35" t="n">
+        <v>32977.99</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>120.87</v>
+      </c>
+      <c r="J35" t="n">
+        <v>34206.21</v>
+      </c>
+      <c r="K35" t="n">
+        <v>-1228.22</v>
+      </c>
+      <c r="L35" t="n">
+        <v>-0.037244</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>6</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>XOP</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>189</v>
+      </c>
+      <c r="F36" t="n">
+        <v>174.13</v>
+      </c>
+      <c r="G36" t="n">
+        <v>32910.57</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>163.99</v>
+      </c>
+      <c r="J36" t="n">
+        <v>30994.11</v>
+      </c>
+      <c r="K36" t="n">
+        <v>1916.46</v>
+      </c>
+      <c r="L36" t="n">
+        <v>0.058232</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>6</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>64</v>
+      </c>
+      <c r="F37" t="n">
+        <v>508.52</v>
+      </c>
+      <c r="G37" t="n">
+        <v>32545.28</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>569.08</v>
+      </c>
+      <c r="J37" t="n">
+        <v>36421.12</v>
+      </c>
+      <c r="K37" t="n">
+        <v>-3875.84</v>
+      </c>
+      <c r="L37" t="n">
+        <v>-0.119091</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>7</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>XLI</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>189</v>
+      </c>
+      <c r="F38" t="n">
+        <v>173.13</v>
+      </c>
+      <c r="G38" t="n">
+        <v>32721.57</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>171.21</v>
+      </c>
+      <c r="J38" t="n">
+        <v>32358.69</v>
+      </c>
+      <c r="K38" t="n">
+        <v>-362.88</v>
+      </c>
+      <c r="L38" t="n">
+        <v>-0.01109</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>7</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>SMH</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>54</v>
+      </c>
+      <c r="F39" t="n">
+        <v>598.9299999999999</v>
+      </c>
+      <c r="G39" t="n">
+        <v>32342.22</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>575.525</v>
+      </c>
+      <c r="J39" t="n">
+        <v>31078.35</v>
+      </c>
+      <c r="K39" t="n">
+        <v>-1263.87</v>
+      </c>
+      <c r="L39" t="n">
+        <v>-0.039078</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>7</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>KBE</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>517</v>
+      </c>
+      <c r="F40" t="n">
+        <v>63.49</v>
+      </c>
+      <c r="G40" t="n">
+        <v>32824.33</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>65.69</v>
+      </c>
+      <c r="J40" t="n">
+        <v>33961.73</v>
+      </c>
+      <c r="K40" t="n">
+        <v>1137.4</v>
+      </c>
+      <c r="L40" t="n">
+        <v>0.034651</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>7</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>XLE</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>584</v>
+      </c>
+      <c r="F41" t="n">
+        <v>56.29</v>
+      </c>
+      <c r="G41" t="n">
+        <v>32873.36</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>58.8759</v>
+      </c>
+      <c r="J41" t="n">
+        <v>34383.53</v>
+      </c>
+      <c r="K41" t="n">
+        <v>-1510.17</v>
+      </c>
+      <c r="L41" t="n">
+        <v>-0.045939</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>7</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>ITA</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>139</v>
+      </c>
+      <c r="F42" t="n">
+        <v>235.44</v>
+      </c>
+      <c r="G42" t="n">
+        <v>32726.16</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>227.07</v>
+      </c>
+      <c r="J42" t="n">
+        <v>31562.73</v>
+      </c>
+      <c r="K42" t="n">
+        <v>1163.43</v>
+      </c>
+      <c r="L42" t="n">
+        <v>0.03555</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>7</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>IGV</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>323</v>
+      </c>
+      <c r="F43" t="n">
+        <v>101.66</v>
+      </c>
+      <c r="G43" t="n">
+        <v>32836.18</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>92.91</v>
+      </c>
+      <c r="J43" t="n">
+        <v>30009.93</v>
+      </c>
+      <c r="K43" t="n">
+        <v>2826.25</v>
+      </c>
+      <c r="L43" t="n">
+        <v>0.08607099999999999</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>8</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>XLY</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>294</v>
+      </c>
+      <c r="F44" t="n">
+        <v>114.005</v>
+      </c>
+      <c r="G44" t="n">
+        <v>33517.47</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>116.6</v>
+      </c>
+      <c r="J44" t="n">
+        <v>34280.4</v>
+      </c>
+      <c r="K44" t="n">
+        <v>762.9299999999999</v>
+      </c>
+      <c r="L44" t="n">
+        <v>0.022762</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>8</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>SMH</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>58</v>
+      </c>
+      <c r="F45" t="n">
+        <v>575.525</v>
+      </c>
+      <c r="G45" t="n">
+        <v>33380.45</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>619.96</v>
+      </c>
+      <c r="J45" t="n">
+        <v>35957.68</v>
+      </c>
+      <c r="K45" t="n">
+        <v>2577.23</v>
+      </c>
+      <c r="L45" t="n">
+        <v>0.077208</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>8</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>XLC</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>300</v>
+      </c>
+      <c r="F46" t="n">
+        <v>111.71</v>
+      </c>
+      <c r="G46" t="n">
+        <v>33513</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>111.65</v>
+      </c>
+      <c r="J46" t="n">
+        <v>33495</v>
+      </c>
+      <c r="K46" t="n">
+        <v>-18</v>
+      </c>
+      <c r="L46" t="n">
+        <v>-0.000537</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>8</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>XLV</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>218</v>
+      </c>
+      <c r="F47" t="n">
+        <v>153.61</v>
+      </c>
+      <c r="G47" t="n">
+        <v>33486.98</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>153.81</v>
+      </c>
+      <c r="J47" t="n">
+        <v>33530.58</v>
+      </c>
+      <c r="K47" t="n">
+        <v>-43.6</v>
+      </c>
+      <c r="L47" t="n">
+        <v>-0.001302</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>8</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>KRE</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>465</v>
+      </c>
+      <c r="F48" t="n">
+        <v>72.05500000000001</v>
+      </c>
+      <c r="G48" t="n">
+        <v>33505.58</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>73.41</v>
+      </c>
+      <c r="J48" t="n">
+        <v>34135.65</v>
+      </c>
+      <c r="K48" t="n">
+        <v>-630.0700000000001</v>
+      </c>
+      <c r="L48" t="n">
+        <v>-0.018805</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>8</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>SOXX</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>61</v>
+      </c>
+      <c r="F49" t="n">
+        <v>546.5650000000001</v>
+      </c>
+      <c r="G49" t="n">
+        <v>33340.47</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>596.25</v>
+      </c>
+      <c r="J49" t="n">
+        <v>36371.25</v>
+      </c>
+      <c r="K49" t="n">
+        <v>-3030.78</v>
+      </c>
+      <c r="L49" t="n">
+        <v>-0.090904</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>9</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>XLC</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>299</v>
+      </c>
+      <c r="F50" t="n">
+        <v>111.65</v>
+      </c>
+      <c r="G50" t="n">
+        <v>33383.35</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>9</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>IHI</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>673</v>
+      </c>
+      <c r="F51" t="n">
+        <v>49.67</v>
+      </c>
+      <c r="G51" t="n">
+        <v>33427.91</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>9</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>XLY</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>286</v>
+      </c>
+      <c r="F52" t="n">
+        <v>116.6</v>
+      </c>
+      <c r="G52" t="n">
+        <v>33347.6</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>9</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>XBI</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>250</v>
+      </c>
+      <c r="F53" t="n">
+        <v>133.79</v>
+      </c>
+      <c r="G53" t="n">
+        <v>33447.5</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>9</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>KRE</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>455</v>
+      </c>
+      <c r="F54" t="n">
+        <v>73.41</v>
+      </c>
+      <c r="G54" t="n">
+        <v>33401.55</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>9</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>KBE</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>499</v>
+      </c>
+      <c r="F55" t="n">
+        <v>66.94</v>
+      </c>
+      <c r="G55" t="n">
+        <v>33403.06</v>
       </c>
     </row>
   </sheetData>
@@ -687,11 +2895,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
@@ -742,6 +2950,246 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-1771.22</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-0.008462000000000001</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-1771.22</v>
+      </c>
+      <c r="H2" t="n">
+        <v>-0.008292000000000001</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-5739.56</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-0.027724</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-7510.78</v>
+      </c>
+      <c r="H3" t="n">
+        <v>-0.035441</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-2758.47</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-0.013711</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-10269.25</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-0.049094</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>9</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-3813.18</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-0.018928</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-14082.43</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-0.068343</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-115.27</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-0.000583</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-14197.7</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-0.070144</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>15</v>
+      </c>
+      <c r="E7" t="n">
+        <v>258.56</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.001309</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-13939.14</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-0.069317</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1990.17</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.010137</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-11948.97</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-0.05876</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-382.29</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-0.001904</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-12331.26</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-0.060095</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>